<commit_message>
chronology pdf exportaion done !
</commit_message>
<xml_diff>
--- a/mock_e2e_project/7. Chronology/Master/Ladder_Chronology.xlsx
+++ b/mock_e2e_project/7. Chronology/Master/Ladder_Chronology.xlsx
@@ -9,7 +9,9 @@
   <sheets>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sheet" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
-  <definedNames/>
+  <definedNames>
+    <definedName name="_xlnm.Print_Area" localSheetId="0">'Sheet'!$A$1:$P$42</definedName>
+  </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
 </file>
@@ -17,10 +19,18 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="1">
+  <fonts count="2">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
+      <color theme="1"/>
+      <sz val="11"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <b val="1"/>
       <color theme="1"/>
       <sz val="11"/>
       <scheme val="minor"/>
@@ -46,8 +56,15 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="1">
+  <cellXfs count="4">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -420,100 +437,343 @@
     <row r="2"/>
     <row r="3"/>
     <row r="4"/>
-    <row r="5"/>
-    <row r="6"/>
-    <row r="7"/>
-    <row r="8"/>
-    <row r="9"/>
-    <row r="10"/>
-    <row r="11"/>
-    <row r="12"/>
-    <row r="13"/>
+    <row r="5">
+      <c r="A5" s="1" t="inlineStr">
+        <is>
+          <t>Product Series:</t>
+        </is>
+      </c>
+      <c r="B5" s="1" t="inlineStr">
+        <is>
+          <t>LPRS480</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr"/>
+      <c r="D5" t="inlineStr"/>
+      <c r="E5" t="inlineStr"/>
+      <c r="F5" t="inlineStr"/>
+      <c r="G5" t="inlineStr"/>
+      <c r="H5" t="inlineStr"/>
+      <c r="I5" t="inlineStr"/>
+      <c r="J5" t="inlineStr"/>
+      <c r="K5" t="inlineStr"/>
+      <c r="L5" t="inlineStr"/>
+      <c r="M5" t="inlineStr"/>
+      <c r="N5" t="inlineStr"/>
+      <c r="O5" t="inlineStr"/>
+      <c r="P5" t="inlineStr"/>
+    </row>
+    <row r="6">
+      <c r="A6" s="1" t="inlineStr">
+        <is>
+          <t>Applicable Products:</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr"/>
+      <c r="C6" t="inlineStr"/>
+      <c r="D6" t="inlineStr"/>
+      <c r="E6" t="inlineStr"/>
+      <c r="F6" t="inlineStr"/>
+      <c r="G6" t="inlineStr"/>
+      <c r="H6" t="inlineStr"/>
+      <c r="I6" t="inlineStr"/>
+      <c r="J6" t="inlineStr"/>
+      <c r="K6" t="inlineStr"/>
+      <c r="L6" t="inlineStr"/>
+      <c r="M6" t="inlineStr"/>
+      <c r="N6" t="inlineStr"/>
+      <c r="O6" t="inlineStr"/>
+      <c r="P6" t="inlineStr"/>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr"/>
+      <c r="B7" t="inlineStr"/>
+      <c r="C7" t="inlineStr"/>
+      <c r="D7" t="inlineStr"/>
+      <c r="E7" t="inlineStr"/>
+      <c r="F7" t="inlineStr"/>
+      <c r="G7" t="inlineStr"/>
+      <c r="H7" t="inlineStr"/>
+      <c r="I7" t="inlineStr"/>
+      <c r="J7" t="inlineStr"/>
+      <c r="K7" t="inlineStr"/>
+      <c r="L7" t="inlineStr"/>
+      <c r="M7" t="inlineStr"/>
+      <c r="N7" t="inlineStr"/>
+      <c r="O7" t="inlineStr"/>
+      <c r="P7" t="inlineStr"/>
+    </row>
+    <row r="8">
+      <c r="A8" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="B8" s="3" t="inlineStr">
+        <is>
+          <t>LRPS480-24-CE</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr"/>
+      <c r="D8" t="inlineStr"/>
+      <c r="E8" t="inlineStr"/>
+      <c r="F8" t="inlineStr"/>
+      <c r="G8" t="inlineStr"/>
+      <c r="H8" t="inlineStr"/>
+      <c r="I8" t="inlineStr"/>
+      <c r="J8" t="inlineStr"/>
+      <c r="K8" t="inlineStr"/>
+      <c r="L8" t="inlineStr"/>
+      <c r="M8" t="inlineStr"/>
+      <c r="N8" t="inlineStr"/>
+      <c r="O8" t="inlineStr"/>
+      <c r="P8" t="inlineStr"/>
+    </row>
+    <row r="9">
+      <c r="A9" s="2" t="n">
+        <v>2</v>
+      </c>
+      <c r="B9" s="3" t="inlineStr">
+        <is>
+          <t>LRPS480-12-CE</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr"/>
+      <c r="D9" t="inlineStr"/>
+      <c r="E9" t="inlineStr"/>
+      <c r="F9" t="inlineStr"/>
+      <c r="G9" t="inlineStr"/>
+      <c r="H9" t="inlineStr"/>
+      <c r="I9" t="inlineStr"/>
+      <c r="J9" t="inlineStr"/>
+      <c r="K9" t="inlineStr"/>
+      <c r="L9" t="inlineStr"/>
+      <c r="M9" t="inlineStr"/>
+      <c r="N9" t="inlineStr"/>
+      <c r="O9" t="inlineStr"/>
+      <c r="P9" t="inlineStr"/>
+    </row>
+    <row r="10">
+      <c r="A10" s="2" t="n">
+        <v>3</v>
+      </c>
+      <c r="B10" s="3" t="inlineStr">
+        <is>
+          <t>LRPS480-05-CE</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr"/>
+      <c r="D10" t="inlineStr"/>
+      <c r="E10" t="inlineStr"/>
+      <c r="F10" t="inlineStr"/>
+      <c r="G10" t="inlineStr"/>
+      <c r="H10" t="inlineStr"/>
+      <c r="I10" t="inlineStr"/>
+      <c r="J10" t="inlineStr"/>
+      <c r="K10" t="inlineStr"/>
+      <c r="L10" t="inlineStr"/>
+      <c r="M10" t="inlineStr"/>
+      <c r="N10" t="inlineStr"/>
+      <c r="O10" t="inlineStr"/>
+      <c r="P10" t="inlineStr"/>
+    </row>
+    <row r="11">
+      <c r="A11" s="2" t="n">
+        <v>4</v>
+      </c>
+      <c r="B11" s="3" t="inlineStr">
+        <is>
+          <t>LRPS480-24-CE</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr"/>
+      <c r="D11" t="inlineStr"/>
+      <c r="E11" t="inlineStr"/>
+      <c r="F11" t="inlineStr"/>
+      <c r="G11" t="inlineStr"/>
+      <c r="H11" t="inlineStr"/>
+      <c r="I11" t="inlineStr"/>
+      <c r="J11" t="inlineStr"/>
+      <c r="K11" t="inlineStr"/>
+      <c r="L11" t="inlineStr"/>
+      <c r="M11" t="inlineStr"/>
+      <c r="N11" t="inlineStr"/>
+      <c r="O11" t="inlineStr"/>
+      <c r="P11" t="inlineStr"/>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr"/>
+      <c r="B12" t="inlineStr"/>
+      <c r="C12" t="inlineStr"/>
+      <c r="D12" t="inlineStr"/>
+      <c r="E12" t="inlineStr"/>
+      <c r="F12" t="inlineStr"/>
+      <c r="G12" t="inlineStr"/>
+      <c r="H12" t="inlineStr"/>
+      <c r="I12" t="inlineStr"/>
+      <c r="J12" t="inlineStr"/>
+      <c r="K12" t="inlineStr"/>
+      <c r="L12" t="inlineStr"/>
+      <c r="M12" t="inlineStr"/>
+      <c r="N12" t="inlineStr"/>
+      <c r="O12" t="inlineStr"/>
+      <c r="P12" t="inlineStr"/>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>Serial No.</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>Source Code Path</t>
+        </is>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>Bin File Name</t>
+        </is>
+      </c>
+      <c r="D13" t="inlineStr">
+        <is>
+          <t>CRC</t>
+        </is>
+      </c>
+      <c r="E13" t="inlineStr">
+        <is>
+          <t>Ladder Version No.</t>
+        </is>
+      </c>
+      <c r="F13" t="inlineStr">
+        <is>
+          <t>Reason For Upgrade</t>
+        </is>
+      </c>
+      <c r="G13" t="inlineStr">
+        <is>
+          <t>Testing Stage</t>
+        </is>
+      </c>
+      <c r="H13" t="inlineStr">
+        <is>
+          <t>PLC Model</t>
+        </is>
+      </c>
+      <c r="I13" t="inlineStr">
+        <is>
+          <t>Selpro Version &amp; Path</t>
+        </is>
+      </c>
+      <c r="J13" t="inlineStr">
+        <is>
+          <t>Bootloader Version</t>
+        </is>
+      </c>
+      <c r="K13" t="inlineStr">
+        <is>
+          <t>Release Date</t>
+        </is>
+      </c>
+      <c r="L13" t="inlineStr">
+        <is>
+          <t>Released By</t>
+        </is>
+      </c>
+      <c r="M13" t="inlineStr">
+        <is>
+          <t>Ladder Release-To Production</t>
+        </is>
+      </c>
+      <c r="N13" t="inlineStr">
+        <is>
+          <t>Operator Procedure Modification</t>
+        </is>
+      </c>
+      <c r="O13" t="inlineStr">
+        <is>
+          <t>Automation Set Up Modification</t>
+        </is>
+      </c>
+      <c r="P13" t="inlineStr">
+        <is>
+          <t>Tested By</t>
+        </is>
+      </c>
+    </row>
     <row r="14">
-      <c r="A14" t="inlineStr">
-        <is>
-          <t>Serial No.</t>
-        </is>
+      <c r="A14" t="n">
+        <v>25</v>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>Source Code Path</t>
+          <t>C:\Users\SM 464\Desktop\Operational Package Validator\ProjectValidator\mock_e2e_project\2. Bin File\Master\FW_V1.23.bin</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>Bin File Name</t>
+          <t>FW_V1.23.bin</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>CRC</t>
+          <t>A3F91C7E</t>
         </is>
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>Ladder Version No.</t>
+          <t>V1.23</t>
         </is>
       </c>
       <c r="F14" t="inlineStr">
         <is>
-          <t>Reason For Upgrade</t>
+          <t>UI polish final</t>
         </is>
       </c>
       <c r="G14" t="inlineStr">
         <is>
-          <t>Testing Stage</t>
+          <t>Master</t>
         </is>
       </c>
       <c r="H14" t="inlineStr">
         <is>
-          <t>PLC Model</t>
-        </is>
-      </c>
-      <c r="I14" t="inlineStr">
-        <is>
-          <t>Selpro Version &amp; Path</t>
-        </is>
-      </c>
-      <c r="J14" t="inlineStr">
-        <is>
-          <t>Bootloader Version</t>
-        </is>
-      </c>
+          <t>FW</t>
+        </is>
+      </c>
+      <c r="I14" t="inlineStr"/>
+      <c r="J14" t="inlineStr"/>
       <c r="K14" t="inlineStr">
         <is>
-          <t>Release Date</t>
+          <t>06/08/2026</t>
         </is>
       </c>
       <c r="L14" t="inlineStr">
         <is>
-          <t>Released By</t>
+          <t>User</t>
         </is>
       </c>
       <c r="M14" t="inlineStr">
         <is>
-          <t>Ladder Release-To Production</t>
+          <t>Yes</t>
         </is>
       </c>
       <c r="N14" t="inlineStr">
         <is>
-          <t>Operator Procedure Modification</t>
+          <t>No</t>
         </is>
       </c>
       <c r="O14" t="inlineStr">
         <is>
-          <t>Automation Set Up Modification</t>
+          <t>No</t>
         </is>
       </c>
       <c r="P14" t="inlineStr">
         <is>
-          <t>Tested By</t>
+          <t>QA</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="n">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="B15" t="inlineStr">
         <is>
@@ -525,13 +785,11 @@
           <t>FW_V1.23.bin</t>
         </is>
       </c>
-      <c r="D15" t="inlineStr"/>
       <c r="E15" t="inlineStr">
         <is>
           <t>V1.23</t>
         </is>
       </c>
-      <c r="F15" t="inlineStr"/>
       <c r="G15" t="inlineStr">
         <is>
           <t>Master</t>
@@ -542,7 +800,6 @@
           <t>FW</t>
         </is>
       </c>
-      <c r="I15" t="inlineStr"/>
       <c r="J15" t="inlineStr">
         <is>
           <t>V1.23</t>
@@ -553,15 +810,10 @@
           <t>05/08/2026</t>
         </is>
       </c>
-      <c r="L15" t="inlineStr"/>
-      <c r="M15" t="inlineStr"/>
-      <c r="N15" t="inlineStr"/>
-      <c r="O15" t="inlineStr"/>
-      <c r="P15" t="inlineStr"/>
     </row>
     <row r="16">
       <c r="A16" t="n">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="B16" t="inlineStr">
         <is>
@@ -601,7 +853,7 @@
     </row>
     <row r="17">
       <c r="A17" t="n">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="B17" t="inlineStr">
         <is>
@@ -641,7 +893,7 @@
     </row>
     <row r="18">
       <c r="A18" t="n">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="B18" t="inlineStr">
         <is>
@@ -681,7 +933,7 @@
     </row>
     <row r="19">
       <c r="A19" t="n">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="B19" t="inlineStr">
         <is>
@@ -721,7 +973,7 @@
     </row>
     <row r="20">
       <c r="A20" t="n">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="B20" t="inlineStr">
         <is>
@@ -761,7 +1013,7 @@
     </row>
     <row r="21">
       <c r="A21" t="n">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="B21" t="inlineStr">
         <is>
@@ -801,7 +1053,7 @@
     </row>
     <row r="22">
       <c r="A22" t="n">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="B22" t="inlineStr">
         <is>
@@ -841,7 +1093,7 @@
     </row>
     <row r="23">
       <c r="A23" t="n">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="B23" t="inlineStr">
         <is>
@@ -881,7 +1133,7 @@
     </row>
     <row r="24">
       <c r="A24" t="n">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="B24" t="inlineStr">
         <is>
@@ -921,7 +1173,7 @@
     </row>
     <row r="25">
       <c r="A25" t="n">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="B25" t="inlineStr">
         <is>
@@ -961,7 +1213,7 @@
     </row>
     <row r="26">
       <c r="A26" t="n">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="B26" t="inlineStr">
         <is>
@@ -1001,7 +1253,7 @@
     </row>
     <row r="27">
       <c r="A27" t="n">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="B27" t="inlineStr">
         <is>
@@ -1041,7 +1293,7 @@
     </row>
     <row r="28">
       <c r="A28" t="n">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="B28" t="inlineStr">
         <is>
@@ -1081,7 +1333,7 @@
     </row>
     <row r="29">
       <c r="A29" t="n">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="B29" t="inlineStr">
         <is>
@@ -1121,7 +1373,7 @@
     </row>
     <row r="30">
       <c r="A30" t="n">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="B30" t="inlineStr">
         <is>
@@ -1161,7 +1413,7 @@
     </row>
     <row r="31">
       <c r="A31" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="B31" t="inlineStr">
         <is>
@@ -1201,7 +1453,7 @@
     </row>
     <row r="32">
       <c r="A32" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="B32" t="inlineStr">
         <is>
@@ -1241,7 +1493,7 @@
     </row>
     <row r="33">
       <c r="A33" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="B33" t="inlineStr">
         <is>
@@ -1281,7 +1533,7 @@
     </row>
     <row r="34">
       <c r="A34" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="B34" t="inlineStr">
         <is>
@@ -1321,7 +1573,7 @@
     </row>
     <row r="35">
       <c r="A35" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="B35" t="inlineStr">
         <is>
@@ -1361,7 +1613,7 @@
     </row>
     <row r="36">
       <c r="A36" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="B36" t="inlineStr">
         <is>
@@ -1401,45 +1653,48 @@
     </row>
     <row r="37">
       <c r="A37" t="n">
+        <v>2</v>
+      </c>
+      <c r="B37" t="inlineStr">
+        <is>
+          <t>C:\Path\V1.01</t>
+        </is>
+      </c>
+      <c r="C37" t="inlineStr">
+        <is>
+          <t>FW_V1.01.bin</t>
+        </is>
+      </c>
+      <c r="D37" t="inlineStr">
+        <is>
+          <t>ABCD1234</t>
+        </is>
+      </c>
+      <c r="E37" t="inlineStr">
+        <is>
+          <t>V1.01</t>
+        </is>
+      </c>
+      <c r="F37" t="inlineStr">
+        <is>
+          <t>Release</t>
+        </is>
+      </c>
+      <c r="G37" t="inlineStr">
+        <is>
+          <t>Production</t>
+        </is>
+      </c>
+      <c r="H37" t="inlineStr">
+        <is>
+          <t>MODEL-X</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" t="n">
         <v>1</v>
       </c>
-      <c r="B37" t="inlineStr">
-        <is>
-          <t>C:\Path\V1.01</t>
-        </is>
-      </c>
-      <c r="C37" t="inlineStr">
-        <is>
-          <t>FW_V1.01.bin</t>
-        </is>
-      </c>
-      <c r="D37" t="inlineStr">
-        <is>
-          <t>ABCD1234</t>
-        </is>
-      </c>
-      <c r="E37" t="inlineStr">
-        <is>
-          <t>V1.01</t>
-        </is>
-      </c>
-      <c r="F37" t="inlineStr">
-        <is>
-          <t>Release</t>
-        </is>
-      </c>
-      <c r="G37" t="inlineStr">
-        <is>
-          <t>Production</t>
-        </is>
-      </c>
-      <c r="H37" t="inlineStr">
-        <is>
-          <t>MODEL-X</t>
-        </is>
-      </c>
-    </row>
-    <row r="38">
       <c r="B38" t="inlineStr">
         <is>
           <t>Instructions</t>
@@ -1458,8 +1713,8 @@
     </row>
   </sheetData>
   <mergeCells count="2">
-    <mergeCell ref="B39:D39"/>
-    <mergeCell ref="B38:P38"/>
+    <mergeCell ref="B40:D40"/>
+    <mergeCell ref="B39:P39"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>